<commit_message>
Controle de fraudes, reunião de gerentes e disparos automáticos
- Trilha de auditoria: dado já recebido que muda depois fica registrado
  (quem, quando, antes/depois, impacto), com gravidade pela idade do dia;
  a conferência do envio avisa o gerente e a Central recebe um alerta só.
- Tela 🛡️ Auditoria com os cruzamentos: LMC, carga sem nota, nota sem
  entrada, nota repetida, valor de nota, custo médio, abaixo do custo e
  números redondos.
- Tela 📋 Reunião de Gerentes: placar com metas, pauta por gerente e ficha
  para imprimir; só as exceções ficam coloridas.
- B2 Assistente: disparos por horário, na chegada dos dados e cobrança com
  horário limite, para pessoas e grupos do Telegram; --chegada no Actions.
- Demonstração com as situações plantadas e o exemplo ALTERADA.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/b2_bonsucesso/B2 Bonsucesso 09-2026.xlsx
+++ b/data/b2_bonsucesso/B2 Bonsucesso 09-2026.xlsx
@@ -14,7 +14,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'MOVIMENTO DIÁRIO'!$A$1:$H$109</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'COMPRAS'!$A$1:$G$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'COMPRAS'!$A$1:$G$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'DESPESAS'!$A$1:$D$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3737,7 +3737,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3977,28 +3977,28 @@
     </row>
     <row r="9">
       <c r="A9" s="12" t="n">
-        <v>46277</v>
+        <v>46279</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Gasolina Comum</t>
+          <t>Gasolina Aditivada</t>
         </is>
       </c>
       <c r="C9" s="13" t="n">
-        <v>35000</v>
+        <v>10000</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>5.7605</v>
+        <v>5.8885</v>
       </c>
       <c r="E9" s="17" t="n">
-        <v>201617.45</v>
+        <v>58884.6</v>
       </c>
       <c r="F9" t="n">
-        <v>148785</v>
+        <v>148798</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Distribuidora Alfa</t>
+          <t>Distribuidora Paraná</t>
         </is>
       </c>
     </row>
@@ -4008,20 +4008,20 @@
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>Gasolina Aditivada</t>
+          <t>Diesel S10</t>
         </is>
       </c>
       <c r="C10" s="9" t="n">
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="D10" s="10" t="n">
-        <v>5.8885</v>
+        <v>5.8259</v>
       </c>
       <c r="E10" s="16" t="n">
-        <v>58884.6</v>
+        <v>87389.2</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>148798</v>
+        <v>148809</v>
       </c>
       <c r="G10" s="8" t="inlineStr">
         <is>
@@ -4031,82 +4031,82 @@
     </row>
     <row r="11">
       <c r="A11" s="12" t="n">
-        <v>46279</v>
+        <v>46281</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Diesel S10</t>
+          <t>Etanol</t>
         </is>
       </c>
       <c r="C11" s="13" t="n">
         <v>15000</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>5.8259</v>
+        <v>4</v>
       </c>
       <c r="E11" s="17" t="n">
-        <v>87389.2</v>
+        <v>59999.38</v>
       </c>
       <c r="F11" t="n">
-        <v>148809</v>
+        <v>148819</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Distribuidora Paraná</t>
+          <t>Distribuidora Alfa</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="n">
-        <v>46281</v>
+        <v>46284</v>
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>Etanol</t>
+          <t>Gasolina Comum</t>
         </is>
       </c>
       <c r="C12" s="9" t="n">
-        <v>15000</v>
+        <v>35000</v>
       </c>
       <c r="D12" s="10" t="n">
-        <v>4</v>
+        <v>5.751</v>
       </c>
       <c r="E12" s="16" t="n">
-        <v>59999.38</v>
+        <v>201284.47</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>148819</v>
+        <v>148822</v>
       </c>
       <c r="G12" s="8" t="inlineStr">
         <is>
-          <t>Distribuidora Alfa</t>
+          <t>Distribuidora Paraná</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="12" t="n">
-        <v>46284</v>
+        <v>46286</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Gasolina Comum</t>
+          <t>Gasolina Aditivada</t>
         </is>
       </c>
       <c r="C13" s="13" t="n">
-        <v>35000</v>
+        <v>10000</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>5.751</v>
+        <v>5.9105</v>
       </c>
       <c r="E13" s="17" t="n">
-        <v>201284.47</v>
+        <v>59105.2</v>
       </c>
       <c r="F13" t="n">
-        <v>148822</v>
+        <v>148844</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Distribuidora Paraná</t>
+          <t>Distribuidora Alfa</t>
         </is>
       </c>
     </row>
@@ -4116,24 +4116,24 @@
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>Gasolina Aditivada</t>
+          <t>Etanol</t>
         </is>
       </c>
       <c r="C14" s="9" t="n">
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="D14" s="10" t="n">
-        <v>5.9105</v>
+        <v>4.0124</v>
       </c>
       <c r="E14" s="16" t="n">
-        <v>59105.2</v>
+        <v>60186.51</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>148844</v>
+        <v>148878</v>
       </c>
       <c r="G14" s="8" t="inlineStr">
         <is>
-          <t>Distribuidora Alfa</t>
+          <t>Distribuidora Sul</t>
         </is>
       </c>
     </row>
@@ -4143,47 +4143,47 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Etanol</t>
+          <t>Diesel S10</t>
         </is>
       </c>
       <c r="C15" s="13" t="n">
         <v>15000</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>4.0124</v>
+        <v>6.1013</v>
       </c>
       <c r="E15" s="17" t="n">
-        <v>60186.51</v>
+        <v>91519.87</v>
       </c>
       <c r="F15" t="n">
-        <v>148878</v>
+        <v>148896</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Distribuidora Sul</t>
+          <t>Distribuidora Paraná</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="n">
-        <v>46286</v>
+        <v>46288</v>
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>Diesel S10</t>
+          <t>Gasolina Comum</t>
         </is>
       </c>
       <c r="C16" s="9" t="n">
-        <v>15000</v>
+        <v>25000</v>
       </c>
       <c r="D16" s="10" t="n">
-        <v>6.1013</v>
+        <v>5.7495</v>
       </c>
       <c r="E16" s="16" t="n">
-        <v>91519.87</v>
+        <v>143736.27</v>
       </c>
       <c r="F16" s="8" t="n">
-        <v>148896</v>
+        <v>148905</v>
       </c>
       <c r="G16" s="8" t="inlineStr">
         <is>
@@ -4193,51 +4193,51 @@
     </row>
     <row r="17">
       <c r="A17" s="12" t="n">
-        <v>46288</v>
+        <v>46290</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Gasolina Comum</t>
+          <t>Diesel S10</t>
         </is>
       </c>
       <c r="C17" s="13" t="n">
-        <v>25000</v>
+        <v>15000</v>
       </c>
       <c r="D17" s="14" t="n">
-        <v>5.7495</v>
+        <v>6.1086</v>
       </c>
       <c r="E17" s="17" t="n">
-        <v>143736.27</v>
+        <v>91629.05</v>
       </c>
       <c r="F17" t="n">
-        <v>148905</v>
+        <v>148937</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Distribuidora Paraná</t>
+          <t>Distribuidora Alfa</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>Diesel S10</t>
+          <t>Etanol</t>
         </is>
       </c>
       <c r="C18" s="9" t="n">
         <v>15000</v>
       </c>
       <c r="D18" s="10" t="n">
-        <v>6.1086</v>
+        <v>3.9914</v>
       </c>
       <c r="E18" s="16" t="n">
-        <v>91629.05</v>
+        <v>59871.34</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>148937</v>
+        <v>148973</v>
       </c>
       <c r="G18" s="8" t="inlineStr">
         <is>
@@ -4245,35 +4245,8 @@
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="12" t="n">
-        <v>46291</v>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Etanol</t>
-        </is>
-      </c>
-      <c r="C19" s="13" t="n">
-        <v>15000</v>
-      </c>
-      <c r="D19" s="14" t="n">
-        <v>3.9914</v>
-      </c>
-      <c r="E19" s="17" t="n">
-        <v>59871.34</v>
-      </c>
-      <c r="F19" t="n">
-        <v>148973</v>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>Distribuidora Alfa</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:G19"/>
+  <autoFilter ref="A1:G18"/>
   <dataValidations count="1">
     <dataValidation sqref="B2:B2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor fora da lista" error="Escolha um item da lista." type="list">
       <formula1>"Gasolina Comum,Gasolina Aditivada,Etanol,Diesel S10"</formula1>

</xml_diff>